<commit_message>
test: add test event to programme Excel
Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/programme.xlsx
+++ b/data/programme.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="308" uniqueCount="161">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="317" uniqueCount="166">
   <si>
     <t>Programme printemps-été 2026</t>
   </si>
@@ -504,6 +504,21 @@
   </si>
   <si>
     <t>30 juillet</t>
+  </si>
+  <si>
+    <t>Août 2026</t>
+  </si>
+  <si>
+    <t>1er août</t>
+  </si>
+  <si>
+    <t>Test pipeline</t>
+  </si>
+  <si>
+    <t>Événement de test — à supprimer</t>
+  </si>
+  <si>
+    <t>Cet événement est un test du pipeline de génération automatique.</t>
   </si>
 </sst>
 </file>
@@ -914,13 +929,13 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:I34"/>
+  <dimension ref="A1:I35"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="18" customWidth="1"/>
@@ -1920,8 +1935,37 @@
         <v>108</v>
       </c>
     </row>
+    <row r="35" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A35" t="s">
+        <v>161</v>
+      </c>
+      <c r="B35" t="s">
+        <v>12</v>
+      </c>
+      <c r="C35" t="s">
+        <v>162</v>
+      </c>
+      <c r="D35" t="s">
+        <v>145</v>
+      </c>
+      <c r="E35" t="s">
+        <v>163</v>
+      </c>
+      <c r="F35" t="s">
+        <v>164</v>
+      </c>
+      <c r="G35" s="1" t="s">
+        <v>165</v>
+      </c>
+      <c r="H35" t="s">
+        <v>24</v>
+      </c>
+      <c r="I35" t="s">
+        <v>32</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
mise à jour du programme
</commit_message>
<xml_diff>
--- a/data/programme.xlsx
+++ b/data/programme.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="279" uniqueCount="160">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="245" uniqueCount="141">
   <si>
     <t xml:space="preserve">Programme printemps-été 2026</t>
   </si>
@@ -56,108 +56,31 @@
     <t xml:space="preserve">Contact</t>
   </si>
   <si>
-    <t xml:space="preserve">Janvier 2026</t>
+    <t xml:space="preserve">Dimanche</t>
+  </si>
+  <si>
+    <t xml:space="preserve">22 février</t>
+  </si>
+  <si>
+    <t xml:space="preserve">14h - 17h</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Atelier avec Florence Sagory, réflexologue esthéticienne</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Atelier cosmétiques au naturel — Crème hydratante au géranium rosat</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Venez créer votre crème hydratante au géranium rosat. L'occasion de passer un dimanche bien-être. Nous finirons par un goûter convivial.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Participation libre</t>
+  </si>
+  <si>
+    <t xml:space="preserve">06 31 50 68 00</t>
   </si>
   <si>
     <t xml:space="preserve">Samedi</t>
-  </si>
-  <si>
-    <t xml:space="preserve">31 janvier</t>
-  </si>
-  <si>
-    <t xml:space="preserve">10h - 13h</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Atelier avec Rose</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Art du mouvement avec la méthode Feldenkrais — Le dos en mouvement !</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Vous souffrez de tensions cervicales, lombalgies, certaines difficultés à se pencher ou tourner la tête. Cet atelier est pour vous ! Lors de cette matinée, vous pratiquerez des mouvements simples, doux et inhabituels : Sentir et développer la richesse des possibilités de notre chaîne vertébrale pour redonner souplesse et vitalité à votre dos. Une invitation à redécouvrir un dos libre, vivant et un quotidien plus fluide !</t>
-  </si>
-  <si>
-    <t xml:space="preserve">35 € + 5 € adhésion annuelle</t>
-  </si>
-  <si>
-    <t xml:space="preserve">rosegiovannini@free.fr — http://www.rosegiovannini.com</t>
-  </si>
-  <si>
-    <t xml:space="preserve">14h - 16h</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1, 2, 3 Sommeil !</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Venez découvrir un système innovant afin d'améliorer votre sommeil !
-Le sommeil, c'est un besoin vital… mais parfois, il nous échappe. Longues nuits sans repos, agitation, pensées qui tournent en boucle… Cela vous parle ?
-Le Sounder Sleep Système, créé par Mickel Grumdman, praticien Feldenkrais, est une technique douce et puissante basée sur la respiration et des mini-mouvements.
-Une présentation claire du système, une pratique guidée de 30 minutes, un moment d'échange convivial autour d'une tisane Herbarius !</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Gratuit</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Février 2026</t>
-  </si>
-  <si>
-    <t xml:space="preserve">14 février</t>
-  </si>
-  <si>
-    <t xml:space="preserve">9h30 - 18h</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Stage avec Florence</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Débuter en permaculture</t>
-  </si>
-  <si>
-    <t xml:space="preserve">À l'issue du stage, vous saurez ce qu'est la permaculture (philosophie et techniques). Vous pourrez mettre en pratique les notions-clés pour transformer votre lieu et installer un jardin en autonomie alimentaire, dans le respect de la Vie.
-C'est un stage pratique… vêtements et chaussures adaptées.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">100 €, incluant le repas et les boissons</t>
-  </si>
-  <si>
-    <t xml:space="preserve">f.goulley@herbarius.net</t>
-  </si>
-  <si>
-    <t xml:space="preserve">21 février</t>
-  </si>
-  <si>
-    <t xml:space="preserve">14h - 17h</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Plessage d'osier</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Venez apprendre à monter une barrière tressée en osier, une cabane pour les enfants et pleins d'autres réalisations ! Vous repartirez avec des branches de saule jaune pour mettre en pratique chez vous.
-Apportez une paire de ciseaux, un sécateur et de bons gants de jardinage.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">35 € — Branches d'osier offertes, ainsi qu'une tisane</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Dimanche</t>
-  </si>
-  <si>
-    <t xml:space="preserve">22 février</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Atelier avec Florence Sagory, réflexologue esthéticienne</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Atelier cosmétiques au naturel — Crème hydratante au géranium rosat</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Venez créer votre crème hydratante au géranium rosat. L'occasion de passer un dimanche bien-être. Nous finirons par un goûter convivial.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Participation libre</t>
-  </si>
-  <si>
-    <t xml:space="preserve">06 31 50 68 00</t>
   </si>
   <si>
     <t xml:space="preserve">28 février</t>
@@ -176,6 +99,9 @@
 En collaboration avec Lamballe Terre et Mer.</t>
   </si>
   <si>
+    <t xml:space="preserve">Gratuit</t>
+  </si>
+  <si>
     <t xml:space="preserve">06.03.43.25.28 ou preventiondechets@lamballe-terre-mer.bzh</t>
   </si>
   <si>
@@ -257,6 +183,9 @@
     <t xml:space="preserve">18 - 19 avril</t>
   </si>
   <si>
+    <t xml:space="preserve">9h30 - 18h</t>
+  </si>
+  <si>
     <t xml:space="preserve">Fête des jardins — Château de Pommorio, Tréveneuc</t>
   </si>
   <si>
@@ -339,6 +268,12 @@
   </si>
   <si>
     <t xml:space="preserve">https://www.arduen.com</t>
+  </si>
+  <si>
+    <t xml:space="preserve">10h - 13h</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Atelier avec Rose</t>
   </si>
   <si>
     <t xml:space="preserve">Art du mouvement — Feldenkrais : L'aisance dans la marche</t>
@@ -489,6 +424,9 @@
   </si>
   <si>
     <t xml:space="preserve">Cycle « Un été en mouvement ! ». Retrouver de l'aisance et de la fluidité dans vos articulations.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">14h - 16h</t>
   </si>
   <si>
     <t xml:space="preserve">Visite guidée — Lamballe Armor</t>
@@ -729,7 +667,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:I34"/>
+  <dimension ref="A1:I1048576"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="18"/>
@@ -773,529 +711,526 @@
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="1" t="s">
+      <c r="B2" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="B2" s="1" t="s">
+      <c r="C2" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="C2" s="1" t="s">
+      <c r="D2" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="D2" s="1" t="s">
+      <c r="E2" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="E2" s="1" t="s">
+      <c r="F2" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="F2" s="1" t="s">
+      <c r="G2" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="G2" s="2" t="s">
+      <c r="H2" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="H2" s="1" t="s">
+      <c r="I2" s="1" t="s">
         <v>18</v>
-      </c>
-      <c r="I2" s="1" t="s">
-        <v>19</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B3" s="1" t="s">
-        <v>12</v>
+        <v>19</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>13</v>
+        <v>20</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>15</v>
+        <v>22</v>
       </c>
       <c r="F3" s="1" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="G3" s="2" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="H3" s="1" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="I3" s="1" t="s">
-        <v>19</v>
+        <v>26</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="1" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>12</v>
+        <v>19</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="F4" s="1" t="s">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="G4" s="2" t="s">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="H4" s="1" t="s">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="I4" s="1" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B5" s="1" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>27</v>
+        <v>37</v>
       </c>
       <c r="F5" s="1" t="s">
-        <v>34</v>
+        <v>38</v>
       </c>
       <c r="G5" s="2" t="s">
-        <v>35</v>
+        <v>39</v>
       </c>
       <c r="H5" s="1" t="s">
-        <v>36</v>
+        <v>40</v>
       </c>
       <c r="I5" s="1" t="s">
-        <v>31</v>
+        <v>41</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B6" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="D6" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="E6" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="F6" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="G6" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="H6" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="I6" s="1" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="B7" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="C7" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="D7" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="E7" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="C6" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="D6" s="1" t="s">
-        <v>33</v>
-      </c>
-      <c r="E6" s="1" t="s">
-        <v>39</v>
-      </c>
-      <c r="F6" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="G6" s="2" t="s">
-        <v>41</v>
-      </c>
-      <c r="H6" s="1" t="s">
-        <v>42</v>
-      </c>
-      <c r="I6" s="1" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B7" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="C7" s="1" t="s">
-        <v>44</v>
-      </c>
-      <c r="D7" s="1" t="s">
+      <c r="F7" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="G7" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="H7" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="I7" s="1" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B8" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="E7" s="1" t="s">
-        <v>46</v>
-      </c>
-      <c r="F7" s="1" t="s">
-        <v>47</v>
-      </c>
-      <c r="G7" s="2" t="s">
-        <v>48</v>
-      </c>
-      <c r="H7" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="I7" s="1" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="1" t="s">
-        <v>50</v>
-      </c>
-      <c r="B8" s="1" t="s">
-        <v>12</v>
-      </c>
       <c r="C8" s="1" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="E8" s="1" t="s">
-        <v>53</v>
+        <v>37</v>
       </c>
       <c r="F8" s="1" t="s">
         <v>54</v>
       </c>
-      <c r="G8" s="2" t="s">
+      <c r="H8" s="1" t="s">
         <v>55</v>
       </c>
-      <c r="H8" s="1" t="s">
+      <c r="I8" s="1" t="s">
         <v>56</v>
-      </c>
-      <c r="I8" s="1" t="s">
-        <v>57</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B9" s="1" t="s">
-        <v>37</v>
+        <v>19</v>
       </c>
       <c r="C9" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="D9" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="E9" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="F9" s="1" t="s">
         <v>58</v>
       </c>
-      <c r="D9" s="1" t="s">
-        <v>59</v>
-      </c>
-      <c r="E9" s="1" t="s">
-        <v>60</v>
-      </c>
-      <c r="F9" s="1" t="s">
-        <v>61</v>
-      </c>
       <c r="G9" s="2" t="s">
-        <v>62</v>
+        <v>32</v>
       </c>
       <c r="H9" s="1" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="I9" s="1" t="s">
-        <v>64</v>
+        <v>34</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B10" s="1" t="s">
-        <v>12</v>
+        <v>45</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>65</v>
+        <v>59</v>
       </c>
       <c r="D10" s="1" t="s">
-        <v>45</v>
+        <v>60</v>
       </c>
       <c r="E10" s="1" t="s">
-        <v>46</v>
+        <v>37</v>
       </c>
       <c r="F10" s="1" t="s">
-        <v>66</v>
-      </c>
-      <c r="G10" s="2" t="s">
-        <v>48</v>
+        <v>61</v>
       </c>
       <c r="H10" s="1" t="s">
-        <v>23</v>
+        <v>40</v>
       </c>
       <c r="I10" s="1" t="s">
-        <v>49</v>
+        <v>62</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="B11" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="C11" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="D11" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="E11" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="F11" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="G11" s="2" t="s">
         <v>67</v>
       </c>
-      <c r="B11" s="1" t="s">
+      <c r="H11" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="I11" s="1" t="s">
         <v>68</v>
-      </c>
-      <c r="C11" s="1" t="s">
-        <v>69</v>
-      </c>
-      <c r="D11" s="1" t="s">
-        <v>70</v>
-      </c>
-      <c r="E11" s="1" t="s">
-        <v>60</v>
-      </c>
-      <c r="F11" s="1" t="s">
-        <v>71</v>
-      </c>
-      <c r="G11" s="2" t="s">
-        <v>72</v>
-      </c>
-      <c r="H11" s="1" t="s">
-        <v>73</v>
-      </c>
-      <c r="I11" s="1" t="s">
-        <v>74</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B12" s="1" t="s">
-        <v>68</v>
+        <v>11</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>75</v>
+        <v>69</v>
       </c>
       <c r="D12" s="1" t="s">
-        <v>26</v>
+        <v>70</v>
       </c>
       <c r="E12" s="1" t="s">
-        <v>60</v>
+        <v>37</v>
       </c>
       <c r="F12" s="1" t="s">
-        <v>76</v>
+        <v>71</v>
+      </c>
+      <c r="G12" s="2" t="s">
+        <v>72</v>
       </c>
       <c r="H12" s="1" t="s">
-        <v>77</v>
+        <v>25</v>
       </c>
       <c r="I12" s="1" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B13" s="1" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>79</v>
+        <v>74</v>
       </c>
       <c r="D13" s="1" t="s">
-        <v>52</v>
+        <v>13</v>
       </c>
       <c r="E13" s="1" t="s">
-        <v>53</v>
+        <v>14</v>
       </c>
       <c r="F13" s="1" t="s">
-        <v>80</v>
+        <v>75</v>
       </c>
       <c r="G13" s="2" t="s">
-        <v>55</v>
+        <v>76</v>
       </c>
       <c r="H13" s="1" t="s">
-        <v>56</v>
+        <v>17</v>
       </c>
       <c r="I13" s="1" t="s">
-        <v>57</v>
+        <v>18</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B14" s="1" t="s">
-        <v>68</v>
+        <v>64</v>
       </c>
       <c r="C14" s="1" t="s">
+        <v>77</v>
+      </c>
+      <c r="D14" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="E14" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="F14" s="1" t="s">
+        <v>78</v>
+      </c>
+      <c r="G14" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="H14" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="I14" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="D14" s="1" t="s">
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B15" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="C15" s="1" t="s">
+        <v>77</v>
+      </c>
+      <c r="D15" s="1" t="s">
         <v>82</v>
       </c>
-      <c r="E14" s="1" t="s">
-        <v>60</v>
-      </c>
-      <c r="F14" s="1" t="s">
+      <c r="E15" s="1" t="s">
         <v>83</v>
       </c>
-      <c r="H14" s="1" t="s">
-        <v>63</v>
-      </c>
-      <c r="I14" s="1" t="s">
+      <c r="F15" s="1" t="s">
         <v>84</v>
       </c>
-    </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="1" t="s">
+      <c r="G15" s="2" t="s">
         <v>85</v>
       </c>
-      <c r="B15" s="1" t="s">
+      <c r="H15" s="1" t="s">
         <v>86</v>
       </c>
-      <c r="C15" s="1" t="s">
+      <c r="I15" s="1" t="s">
         <v>87</v>
-      </c>
-      <c r="D15" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="E15" s="1" t="s">
-        <v>60</v>
-      </c>
-      <c r="F15" s="1" t="s">
-        <v>88</v>
-      </c>
-      <c r="G15" s="2" t="s">
-        <v>89</v>
-      </c>
-      <c r="H15" s="1" t="s">
-        <v>63</v>
-      </c>
-      <c r="I15" s="1" t="s">
-        <v>90</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B16" s="1" t="s">
-        <v>37</v>
+        <v>88</v>
       </c>
       <c r="C16" s="1" t="s">
+        <v>89</v>
+      </c>
+      <c r="D16" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="E16" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="F16" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="G16" s="2" t="s">
         <v>91</v>
       </c>
-      <c r="D16" s="1" t="s">
-        <v>92</v>
-      </c>
-      <c r="E16" s="1" t="s">
-        <v>60</v>
-      </c>
-      <c r="F16" s="1" t="s">
-        <v>93</v>
-      </c>
-      <c r="G16" s="2" t="s">
-        <v>94</v>
-      </c>
       <c r="H16" s="1" t="s">
-        <v>23</v>
+        <v>86</v>
       </c>
       <c r="I16" s="1" t="s">
-        <v>95</v>
+        <v>87</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B17" s="1" t="s">
-        <v>37</v>
+        <v>19</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
       <c r="D17" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="E17" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="F17" s="1" t="s">
+        <v>93</v>
+      </c>
+      <c r="G17" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="H17" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="E17" s="1" t="s">
-        <v>39</v>
-      </c>
-      <c r="F17" s="1" t="s">
-        <v>97</v>
-      </c>
-      <c r="G17" s="2" t="s">
-        <v>98</v>
-      </c>
-      <c r="H17" s="1" t="s">
-        <v>42</v>
-      </c>
       <c r="I17" s="1" t="s">
-        <v>43</v>
+        <v>94</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B18" s="1" t="s">
-        <v>86</v>
+        <v>11</v>
       </c>
       <c r="C18" s="1" t="s">
-        <v>99</v>
+        <v>95</v>
       </c>
       <c r="D18" s="1" t="s">
-        <v>70</v>
+        <v>36</v>
       </c>
       <c r="E18" s="1" t="s">
-        <v>60</v>
+        <v>37</v>
       </c>
       <c r="F18" s="1" t="s">
-        <v>100</v>
+        <v>96</v>
       </c>
       <c r="G18" s="2" t="s">
-        <v>101</v>
+        <v>97</v>
       </c>
       <c r="H18" s="1" t="s">
-        <v>102</v>
+        <v>25</v>
       </c>
       <c r="I18" s="1" t="s">
-        <v>103</v>
+        <v>98</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B19" s="1" t="s">
-        <v>86</v>
+        <v>99</v>
       </c>
       <c r="C19" s="1" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="D19" s="1" t="s">
-        <v>14</v>
+        <v>101</v>
       </c>
       <c r="E19" s="1" t="s">
-        <v>15</v>
+        <v>83</v>
       </c>
       <c r="F19" s="1" t="s">
+        <v>102</v>
+      </c>
+      <c r="G19" s="2" t="s">
+        <v>103</v>
+      </c>
+      <c r="H19" s="1" t="s">
         <v>104</v>
       </c>
-      <c r="G19" s="2" t="s">
-        <v>105</v>
-      </c>
-      <c r="H19" s="1" t="s">
-        <v>106</v>
-      </c>
       <c r="I19" s="1" t="s">
-        <v>107</v>
+        <v>87</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B20" s="1" t="s">
+        <v>99</v>
+      </c>
+      <c r="C20" s="1" t="s">
+        <v>105</v>
+      </c>
+      <c r="D20" s="1" t="s">
+        <v>101</v>
+      </c>
+      <c r="E20" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="F20" s="1" t="s">
+        <v>102</v>
+      </c>
+      <c r="G20" s="2" t="s">
+        <v>103</v>
+      </c>
+      <c r="H20" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="I20" s="1" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="B21" s="1" t="s">
+        <v>107</v>
+      </c>
+      <c r="C21" s="1" t="s">
         <v>108</v>
       </c>
-      <c r="C20" s="1" t="s">
+      <c r="D21" s="1" t="s">
         <v>109</v>
       </c>
-      <c r="D20" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="E20" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="F20" s="1" t="s">
+      <c r="E21" s="1" t="s">
         <v>110</v>
       </c>
-      <c r="G20" s="2" t="s">
+      <c r="F21" s="1" t="s">
         <v>111</v>
       </c>
-      <c r="H20" s="1" t="s">
-        <v>106</v>
-      </c>
-      <c r="I20" s="1" t="s">
-        <v>107</v>
-      </c>
-    </row>
-    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B21" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="C21" s="1" t="s">
+      <c r="G21" s="2" t="s">
         <v>112</v>
       </c>
-      <c r="D21" s="1" t="s">
-        <v>52</v>
-      </c>
-      <c r="E21" s="1" t="s">
-        <v>53</v>
-      </c>
-      <c r="F21" s="1" t="s">
+      <c r="H21" s="1" t="s">
         <v>113</v>
-      </c>
-      <c r="G21" s="2" t="s">
-        <v>55</v>
-      </c>
-      <c r="H21" s="1" t="s">
-        <v>56</v>
       </c>
       <c r="I21" s="1" t="s">
         <v>114</v>
@@ -1303,16 +1238,16 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B22" s="1" t="s">
-        <v>37</v>
+        <v>19</v>
       </c>
       <c r="C22" s="1" t="s">
         <v>115</v>
       </c>
       <c r="D22" s="1" t="s">
-        <v>59</v>
+        <v>21</v>
       </c>
       <c r="E22" s="1" t="s">
-        <v>60</v>
+        <v>22</v>
       </c>
       <c r="F22" s="1" t="s">
         <v>116</v>
@@ -1321,327 +1256,224 @@
         <v>117</v>
       </c>
       <c r="H22" s="1" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="I22" s="1" t="s">
-        <v>118</v>
+        <v>26</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B23" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="C23" s="1" t="s">
+        <v>118</v>
+      </c>
+      <c r="D23" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="E23" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="F23" s="1" t="s">
         <v>119</v>
       </c>
-      <c r="C23" s="1" t="s">
-        <v>120</v>
-      </c>
-      <c r="D23" s="1" t="s">
-        <v>121</v>
-      </c>
-      <c r="E23" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="F23" s="1" t="s">
-        <v>122</v>
-      </c>
       <c r="G23" s="2" t="s">
-        <v>123</v>
+        <v>32</v>
       </c>
       <c r="H23" s="1" t="s">
-        <v>124</v>
+        <v>33</v>
       </c>
       <c r="I23" s="1" t="s">
-        <v>107</v>
+        <v>34</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B24" s="1" t="s">
-        <v>119</v>
+        <v>19</v>
       </c>
       <c r="C24" s="1" t="s">
-        <v>125</v>
+        <v>120</v>
       </c>
       <c r="D24" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="E24" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="F24" s="1" t="s">
         <v>121</v>
       </c>
-      <c r="E24" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="F24" s="1" t="s">
-        <v>122</v>
-      </c>
       <c r="G24" s="2" t="s">
-        <v>123</v>
+        <v>117</v>
       </c>
       <c r="H24" s="1" t="s">
-        <v>124</v>
+        <v>25</v>
       </c>
       <c r="I24" s="1" t="s">
-        <v>107</v>
+        <v>26</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="1" t="s">
+        <v>122</v>
+      </c>
+      <c r="B25" s="1" t="s">
+        <v>99</v>
+      </c>
+      <c r="C25" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="D25" s="1" t="s">
+        <v>124</v>
+      </c>
+      <c r="E25" s="1" t="s">
+        <v>125</v>
+      </c>
+      <c r="F25" s="1" t="s">
         <v>126</v>
       </c>
-      <c r="B25" s="1" t="s">
+      <c r="G25" s="2" t="s">
         <v>127</v>
       </c>
-      <c r="C25" s="1" t="s">
+      <c r="I25" s="1" t="s">
         <v>128</v>
-      </c>
-      <c r="D25" s="1" t="s">
-        <v>129</v>
-      </c>
-      <c r="E25" s="1" t="s">
-        <v>130</v>
-      </c>
-      <c r="F25" s="1" t="s">
-        <v>131</v>
-      </c>
-      <c r="G25" s="2" t="s">
-        <v>132</v>
-      </c>
-      <c r="H25" s="1" t="s">
-        <v>133</v>
-      </c>
-      <c r="I25" s="1" t="s">
-        <v>134</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B26" s="1" t="s">
-        <v>12</v>
+        <v>64</v>
       </c>
       <c r="C26" s="1" t="s">
-        <v>135</v>
+        <v>129</v>
       </c>
       <c r="D26" s="1" t="s">
-        <v>45</v>
+        <v>130</v>
       </c>
       <c r="E26" s="1" t="s">
-        <v>46</v>
+        <v>83</v>
       </c>
       <c r="F26" s="1" t="s">
-        <v>136</v>
+        <v>131</v>
       </c>
       <c r="G26" s="2" t="s">
-        <v>137</v>
+        <v>132</v>
       </c>
       <c r="H26" s="1" t="s">
-        <v>23</v>
+        <v>104</v>
       </c>
       <c r="I26" s="1" t="s">
-        <v>49</v>
+        <v>87</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B27" s="1" t="s">
-        <v>12</v>
+        <v>64</v>
       </c>
       <c r="C27" s="1" t="s">
-        <v>138</v>
+        <v>129</v>
       </c>
       <c r="D27" s="1" t="s">
-        <v>52</v>
+        <v>133</v>
       </c>
       <c r="E27" s="1" t="s">
-        <v>53</v>
+        <v>134</v>
       </c>
       <c r="F27" s="1" t="s">
-        <v>139</v>
+        <v>135</v>
       </c>
       <c r="G27" s="2" t="s">
-        <v>55</v>
+        <v>136</v>
       </c>
       <c r="H27" s="1" t="s">
-        <v>56</v>
+        <v>25</v>
       </c>
       <c r="I27" s="1" t="s">
-        <v>57</v>
+        <v>137</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B28" s="1" t="s">
-        <v>12</v>
+        <v>64</v>
       </c>
       <c r="C28" s="1" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="D28" s="1" t="s">
-        <v>45</v>
+        <v>130</v>
       </c>
       <c r="E28" s="1" t="s">
-        <v>46</v>
+        <v>83</v>
       </c>
       <c r="F28" s="1" t="s">
-        <v>141</v>
+        <v>131</v>
       </c>
       <c r="G28" s="2" t="s">
+        <v>132</v>
+      </c>
+      <c r="H28" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="I28" s="1" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B29" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="C29" s="1" t="s">
+        <v>138</v>
+      </c>
+      <c r="D29" s="1" t="s">
+        <v>133</v>
+      </c>
+      <c r="E29" s="1" t="s">
+        <v>134</v>
+      </c>
+      <c r="F29" s="1" t="s">
+        <v>135</v>
+      </c>
+      <c r="G29" s="2" t="s">
+        <v>139</v>
+      </c>
+      <c r="H29" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="I29" s="1" t="s">
         <v>137</v>
-      </c>
-      <c r="H28" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="I28" s="1" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="1" t="s">
-        <v>142</v>
-      </c>
-      <c r="B29" s="1" t="s">
-        <v>119</v>
-      </c>
-      <c r="C29" s="1" t="s">
-        <v>143</v>
-      </c>
-      <c r="D29" s="1" t="s">
-        <v>144</v>
-      </c>
-      <c r="E29" s="1" t="s">
-        <v>145</v>
-      </c>
-      <c r="F29" s="1" t="s">
-        <v>146</v>
-      </c>
-      <c r="G29" s="2" t="s">
-        <v>147</v>
-      </c>
-      <c r="I29" s="1" t="s">
-        <v>148</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B30" s="1" t="s">
-        <v>86</v>
+        <v>64</v>
       </c>
       <c r="C30" s="1" t="s">
-        <v>149</v>
+        <v>140</v>
       </c>
       <c r="D30" s="1" t="s">
-        <v>150</v>
+        <v>130</v>
       </c>
       <c r="E30" s="1" t="s">
-        <v>15</v>
+        <v>83</v>
       </c>
       <c r="F30" s="1" t="s">
-        <v>151</v>
+        <v>131</v>
       </c>
       <c r="G30" s="2" t="s">
-        <v>152</v>
+        <v>132</v>
       </c>
       <c r="H30" s="1" t="s">
-        <v>124</v>
+        <v>104</v>
       </c>
       <c r="I30" s="1" t="s">
-        <v>107</v>
-      </c>
-    </row>
-    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B31" s="1" t="s">
-        <v>86</v>
-      </c>
-      <c r="C31" s="1" t="s">
-        <v>149</v>
-      </c>
-      <c r="D31" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="E31" s="1" t="s">
-        <v>153</v>
-      </c>
-      <c r="F31" s="1" t="s">
-        <v>154</v>
-      </c>
-      <c r="G31" s="2" t="s">
-        <v>155</v>
-      </c>
-      <c r="H31" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="I31" s="1" t="s">
-        <v>156</v>
-      </c>
-    </row>
-    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B32" s="1" t="s">
-        <v>86</v>
-      </c>
-      <c r="C32" s="1" t="s">
-        <v>157</v>
-      </c>
-      <c r="D32" s="1" t="s">
-        <v>150</v>
-      </c>
-      <c r="E32" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="F32" s="1" t="s">
-        <v>151</v>
-      </c>
-      <c r="G32" s="2" t="s">
-        <v>152</v>
-      </c>
-      <c r="H32" s="1" t="s">
-        <v>124</v>
-      </c>
-      <c r="I32" s="1" t="s">
-        <v>107</v>
-      </c>
-    </row>
-    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B33" s="1" t="s">
-        <v>86</v>
-      </c>
-      <c r="C33" s="1" t="s">
-        <v>157</v>
-      </c>
-      <c r="D33" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="E33" s="1" t="s">
-        <v>153</v>
-      </c>
-      <c r="F33" s="1" t="s">
-        <v>154</v>
-      </c>
-      <c r="G33" s="2" t="s">
-        <v>158</v>
-      </c>
-      <c r="H33" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="I33" s="1" t="s">
-        <v>156</v>
-      </c>
-    </row>
-    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B34" s="1" t="s">
-        <v>86</v>
-      </c>
-      <c r="C34" s="1" t="s">
-        <v>159</v>
-      </c>
-      <c r="D34" s="1" t="s">
-        <v>150</v>
-      </c>
-      <c r="E34" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="F34" s="1" t="s">
-        <v>151</v>
-      </c>
-      <c r="G34" s="2" t="s">
-        <v>152</v>
-      </c>
-      <c r="H34" s="1" t="s">
-        <v>124</v>
-      </c>
-      <c r="I34" s="1" t="s">
-        <v>107</v>
-      </c>
-    </row>
+        <v>87</v>
+      </c>
+    </row>
+    <row r="1048573" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048574" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048575" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048576" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>

<commit_message>
restore initial file for tonight demo
</commit_message>
<xml_diff>
--- a/data/programme.xlsx
+++ b/data/programme.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="229" uniqueCount="136">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="279" uniqueCount="160">
   <si>
     <t xml:space="preserve">Programme printemps-été 2026</t>
   </si>
@@ -56,58 +56,111 @@
     <t xml:space="preserve">Contact</t>
   </si>
   <si>
-    <t xml:space="preserve">Mars 2026</t>
+    <t xml:space="preserve">Janvier 2026</t>
   </si>
   <si>
     <t xml:space="preserve">Samedi</t>
   </si>
   <si>
-    <t xml:space="preserve">21 mars</t>
-  </si>
-  <si>
-    <t xml:space="preserve">14h30 - 17h</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Atelier avec Isabelle</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Élixirs floraux harmonisants du printemps</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Venez à la découverte des Fleurs de Bach !</t>
-  </si>
-  <si>
-    <t xml:space="preserve">25 €</t>
-  </si>
-  <si>
-    <t xml:space="preserve">02.96.32.68.21</t>
+    <t xml:space="preserve">31 janvier</t>
+  </si>
+  <si>
+    <t xml:space="preserve">10h - 13h</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Atelier avec Rose</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Art du mouvement avec la méthode Feldenkrais — Le dos en mouvement !</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Vous souffrez de tensions cervicales, lombalgies, certaines difficultés à se pencher ou tourner la tête. Cet atelier est pour vous ! Lors de cette matinée, vous pratiquerez des mouvements simples, doux et inhabituels : Sentir et développer la richesse des possibilités de notre chaîne vertébrale pour redonner souplesse et vitalité à votre dos. Une invitation à redécouvrir un dos libre, vivant et un quotidien plus fluide !</t>
+  </si>
+  <si>
+    <t xml:space="preserve">35 € + 5 € adhésion annuelle</t>
+  </si>
+  <si>
+    <t xml:space="preserve">rosegiovannini@free.fr — http://www.rosegiovannini.com</t>
+  </si>
+  <si>
+    <t xml:space="preserve">14h - 16h</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1, 2, 3 Sommeil !</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Venez découvrir un système innovant afin d'améliorer votre sommeil !
+Le sommeil, c'est un besoin vital… mais parfois, il nous échappe. Longues nuits sans repos, agitation, pensées qui tournent en boucle… Cela vous parle ?
+Le Sounder Sleep Système, créé par Mickel Grumdman, praticien Feldenkrais, est une technique douce et puissante basée sur la respiration et des mini-mouvements.
+Une présentation claire du système, une pratique guidée de 30 minutes, un moment d'échange convivial autour d'une tisane Herbarius !</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Gratuit</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Février 2026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">14 février</t>
+  </si>
+  <si>
+    <t xml:space="preserve">9h30 - 18h</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Stage avec Florence</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Débuter en permaculture</t>
+  </si>
+  <si>
+    <t xml:space="preserve">À l'issue du stage, vous saurez ce qu'est la permaculture (philosophie et techniques). Vous pourrez mettre en pratique les notions-clés pour transformer votre lieu et installer un jardin en autonomie alimentaire, dans le respect de la Vie.
+C'est un stage pratique… vêtements et chaussures adaptées.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">100 €, incluant le repas et les boissons</t>
+  </si>
+  <si>
+    <t xml:space="preserve">f.goulley@herbarius.net</t>
+  </si>
+  <si>
+    <t xml:space="preserve">21 février</t>
+  </si>
+  <si>
+    <t xml:space="preserve">14h - 17h</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Plessage d'osier</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Venez apprendre à monter une barrière tressée en osier, une cabane pour les enfants et pleins d'autres réalisations ! Vous repartirez avec des branches de saule jaune pour mettre en pratique chez vous.
+Apportez une paire de ciseaux, un sécateur et de bons gants de jardinage.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">35 € — Branches d'osier offertes, ainsi qu'une tisane</t>
   </si>
   <si>
     <t xml:space="preserve">Dimanche</t>
   </si>
   <si>
-    <t xml:space="preserve">22 mars</t>
-  </si>
-  <si>
-    <t xml:space="preserve">9h - 18h</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Exposition</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Herbarius expose au Marché des plantes d'Andel</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Entrée gratuite.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Entrée gratuite</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://comitedesfetesandel.com/</t>
-  </si>
-  <si>
-    <t xml:space="preserve">28 mars</t>
+    <t xml:space="preserve">22 février</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Atelier avec Florence Sagory, réflexologue esthéticienne</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Atelier cosmétiques au naturel — Crème hydratante au géranium rosat</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Venez créer votre crème hydratante au géranium rosat. L'occasion de passer un dimanche bien-être. Nous finirons par un goûter convivial.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Participation libre</t>
+  </si>
+  <si>
+    <t xml:space="preserve">06 31 50 68 00</t>
+  </si>
+  <si>
+    <t xml:space="preserve">28 février</t>
   </si>
   <si>
     <t xml:space="preserve">15h - 17h30</t>
@@ -116,19 +169,67 @@
     <t xml:space="preserve">Atelier avec Florence</t>
   </si>
   <si>
-    <t xml:space="preserve">Jardiner au naturel — Le potager de mars, que semer, comment réussir ?</t>
+    <t xml:space="preserve">Jardiner au naturel — Que semer mois par mois ? Comment réussir ses semis ?</t>
   </si>
   <si>
     <t xml:space="preserve">Venez découvrir comment composter, nourrir le jardin, pailler en réutilisant vos propres ressources (tontes, tailles) !
 En collaboration avec Lamballe Terre et Mer.</t>
   </si>
   <si>
-    <t xml:space="preserve">Gratuit</t>
-  </si>
-  <si>
     <t xml:space="preserve">06.03.43.25.28 ou preventiondechets@lamballe-terre-mer.bzh</t>
   </si>
   <si>
+    <t xml:space="preserve">Mars 2026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">21 mars</t>
+  </si>
+  <si>
+    <t xml:space="preserve">14h30 - 17h</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Atelier avec Isabelle</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Élixirs floraux harmonisants du printemps</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Venez à la découverte des Fleurs de Bach !</t>
+  </si>
+  <si>
+    <t xml:space="preserve">25 €</t>
+  </si>
+  <si>
+    <t xml:space="preserve">02.96.32.68.21</t>
+  </si>
+  <si>
+    <t xml:space="preserve">22 mars</t>
+  </si>
+  <si>
+    <t xml:space="preserve">9h - 18h</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Exposition</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Herbarius expose au Marché des plantes d'Andel</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Entrée gratuite.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Entrée gratuite</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://comitedesfetesandel.com/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">28 mars</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Jardiner au naturel — Le potager de mars, que semer, comment réussir ?</t>
+  </si>
+  <si>
     <t xml:space="preserve">Avril 2026</t>
   </si>
   <si>
@@ -156,9 +257,6 @@
     <t xml:space="preserve">18 - 19 avril</t>
   </si>
   <si>
-    <t xml:space="preserve">9h30 - 18h</t>
-  </si>
-  <si>
     <t xml:space="preserve">Fête des jardins — Château de Pommorio, Tréveneuc</t>
   </si>
   <si>
@@ -222,24 +320,12 @@
     <t xml:space="preserve">10 mai</t>
   </si>
   <si>
-    <t xml:space="preserve">14h - 17h</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Atelier avec Florence Sagory, réflexologue esthéticienne</t>
-  </si>
-  <si>
     <t xml:space="preserve">Atelier cosmétiques au naturel — Huile aux fleurs du jardin</t>
   </si>
   <si>
     <t xml:space="preserve">Venez créer votre huile aux fleurs du jardin qui servira au massage ou à la relaxation. Initiation à la réflexologie fasciale. Nous finirons par un goûter convivial.</t>
   </si>
   <si>
-    <t xml:space="preserve">Participation libre</t>
-  </si>
-  <si>
-    <t xml:space="preserve">06 31 50 68 00</t>
-  </si>
-  <si>
     <t xml:space="preserve">14 mai</t>
   </si>
   <si>
@@ -253,12 +339,6 @@
   </si>
   <si>
     <t xml:space="preserve">https://www.arduen.com</t>
-  </si>
-  <si>
-    <t xml:space="preserve">10h - 13h</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Atelier avec Rose</t>
   </si>
   <si>
     <t xml:space="preserve">Art du mouvement — Feldenkrais : L'aisance dans la marche</t>
@@ -409,9 +489,6 @@
   </si>
   <si>
     <t xml:space="preserve">Cycle « Un été en mouvement ! ». Retrouver de l'aisance et de la fluidité dans vos articulations.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">14h - 16h</t>
   </si>
   <si>
     <t xml:space="preserve">Visite guidée — Lamballe Armor</t>
@@ -652,7 +729,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:I1048576"/>
+  <dimension ref="A1:I34"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="18"/>
@@ -726,106 +803,109 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B3" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="D3" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="C3" s="1" t="s">
+      <c r="E3" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="F3" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="D3" s="1" t="s">
+      <c r="G3" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="E3" s="1" t="s">
+      <c r="H3" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="F3" s="1" t="s">
+      <c r="I3" s="1" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="G3" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="H3" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="I3" s="1" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B4" s="1" t="s">
         <v>12</v>
       </c>
       <c r="C4" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="D4" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="E4" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="F4" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="D4" s="1" t="s">
+      <c r="G4" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="E4" s="1" t="s">
+      <c r="H4" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="F4" s="1" t="s">
+      <c r="I4" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="G4" s="2" t="s">
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B5" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="C5" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="H4" s="1" t="s">
+      <c r="D5" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="I4" s="1" t="s">
+      <c r="E5" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="F5" s="1" t="s">
         <v>34</v>
       </c>
-    </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="1" t="s">
+      <c r="G5" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="B5" s="1" t="s">
+      <c r="H5" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="C5" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="D5" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="E5" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="F5" s="1" t="s">
-        <v>39</v>
-      </c>
-      <c r="G5" s="2" t="s">
-        <v>40</v>
-      </c>
-      <c r="H5" s="1" t="s">
-        <v>41</v>
-      </c>
       <c r="I5" s="1" t="s">
-        <v>42</v>
+        <v>31</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B6" s="1" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="C6" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="D6" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="E6" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="F6" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="G6" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="H6" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="I6" s="1" t="s">
         <v>43</v>
-      </c>
-      <c r="D6" s="1" t="s">
-        <v>44</v>
-      </c>
-      <c r="E6" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="F6" s="1" t="s">
-        <v>45</v>
-      </c>
-      <c r="H6" s="1" t="s">
-        <v>46</v>
-      </c>
-      <c r="I6" s="1" t="s">
-        <v>47</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -833,273 +913,276 @@
         <v>12</v>
       </c>
       <c r="C7" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="D7" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="E7" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="F7" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="G7" s="2" t="s">
         <v>48</v>
       </c>
-      <c r="D7" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="E7" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="F7" s="1" t="s">
+      <c r="H7" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="I7" s="1" t="s">
         <v>49</v>
       </c>
-      <c r="G7" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="H7" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="I7" s="1" t="s">
-        <v>19</v>
-      </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="1" t="s">
+        <v>50</v>
+      </c>
       <c r="B8" s="1" t="s">
-        <v>36</v>
+        <v>12</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="E8" s="1" t="s">
-        <v>23</v>
+        <v>53</v>
       </c>
       <c r="F8" s="1" t="s">
-        <v>52</v>
+        <v>54</v>
+      </c>
+      <c r="G8" s="2" t="s">
+        <v>55</v>
       </c>
       <c r="H8" s="1" t="s">
-        <v>26</v>
+        <v>56</v>
       </c>
       <c r="I8" s="1" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="1" t="s">
-        <v>54</v>
-      </c>
       <c r="B9" s="1" t="s">
-        <v>55</v>
+        <v>37</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>44</v>
+        <v>59</v>
       </c>
       <c r="E9" s="1" t="s">
-        <v>23</v>
+        <v>60</v>
       </c>
       <c r="F9" s="1" t="s">
-        <v>57</v>
+        <v>61</v>
       </c>
       <c r="G9" s="2" t="s">
-        <v>58</v>
+        <v>62</v>
       </c>
       <c r="H9" s="1" t="s">
-        <v>26</v>
+        <v>63</v>
       </c>
       <c r="I9" s="1" t="s">
-        <v>59</v>
+        <v>64</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B10" s="1" t="s">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="C10" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="D10" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="E10" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="F10" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="G10" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="H10" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="I10" s="1" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="B11" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="C11" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="D11" s="1" t="s">
+        <v>70</v>
+      </c>
+      <c r="E11" s="1" t="s">
         <v>60</v>
       </c>
-      <c r="D10" s="1" t="s">
-        <v>61</v>
-      </c>
-      <c r="E10" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="F10" s="1" t="s">
-        <v>62</v>
-      </c>
-      <c r="G10" s="2" t="s">
-        <v>63</v>
-      </c>
-      <c r="H10" s="1" t="s">
-        <v>33</v>
-      </c>
-      <c r="I10" s="1" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B11" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="C11" s="1" t="s">
-        <v>65</v>
-      </c>
-      <c r="D11" s="1" t="s">
-        <v>66</v>
-      </c>
-      <c r="E11" s="1" t="s">
-        <v>67</v>
-      </c>
       <c r="F11" s="1" t="s">
-        <v>68</v>
+        <v>71</v>
       </c>
       <c r="G11" s="2" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="H11" s="1" t="s">
-        <v>70</v>
+        <v>73</v>
       </c>
       <c r="I11" s="1" t="s">
-        <v>71</v>
+        <v>74</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B12" s="1" t="s">
-        <v>55</v>
+        <v>68</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="D12" s="1" t="s">
-        <v>38</v>
+        <v>26</v>
       </c>
       <c r="E12" s="1" t="s">
-        <v>23</v>
+        <v>60</v>
       </c>
       <c r="F12" s="1" t="s">
-        <v>73</v>
-      </c>
-      <c r="G12" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="H12" s="1" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="I12" s="1" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B13" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="C13" s="1" t="s">
+        <v>79</v>
+      </c>
+      <c r="D13" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="E13" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="F13" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="G13" s="2" t="s">
         <v>55</v>
       </c>
-      <c r="C13" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="D13" s="1" t="s">
-        <v>77</v>
-      </c>
-      <c r="E13" s="1" t="s">
-        <v>78</v>
-      </c>
-      <c r="F13" s="1" t="s">
-        <v>79</v>
-      </c>
-      <c r="G13" s="2" t="s">
-        <v>80</v>
-      </c>
       <c r="H13" s="1" t="s">
-        <v>81</v>
+        <v>56</v>
       </c>
       <c r="I13" s="1" t="s">
-        <v>82</v>
+        <v>57</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B14" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="C14" s="1" t="s">
+        <v>81</v>
+      </c>
+      <c r="D14" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="E14" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="F14" s="1" t="s">
         <v>83</v>
       </c>
-      <c r="C14" s="1" t="s">
+      <c r="H14" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="I14" s="1" t="s">
         <v>84</v>
       </c>
-      <c r="D14" s="1" t="s">
-        <v>77</v>
-      </c>
-      <c r="E14" s="1" t="s">
-        <v>78</v>
-      </c>
-      <c r="F14" s="1" t="s">
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="1" t="s">
         <v>85</v>
       </c>
-      <c r="G14" s="2" t="s">
+      <c r="B15" s="1" t="s">
         <v>86</v>
-      </c>
-      <c r="H14" s="1" t="s">
-        <v>81</v>
-      </c>
-      <c r="I14" s="1" t="s">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B15" s="1" t="s">
-        <v>12</v>
       </c>
       <c r="C15" s="1" t="s">
         <v>87</v>
       </c>
       <c r="D15" s="1" t="s">
-        <v>14</v>
+        <v>26</v>
       </c>
       <c r="E15" s="1" t="s">
-        <v>15</v>
+        <v>60</v>
       </c>
       <c r="F15" s="1" t="s">
         <v>88</v>
       </c>
       <c r="G15" s="2" t="s">
-        <v>17</v>
+        <v>89</v>
       </c>
       <c r="H15" s="1" t="s">
-        <v>18</v>
+        <v>63</v>
       </c>
       <c r="I15" s="1" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B16" s="1" t="s">
-        <v>20</v>
+        <v>37</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="D16" s="1" t="s">
-        <v>22</v>
+        <v>92</v>
       </c>
       <c r="E16" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="F16" s="1" t="s">
+        <v>93</v>
+      </c>
+      <c r="G16" s="2" t="s">
+        <v>94</v>
+      </c>
+      <c r="H16" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="F16" s="1" t="s">
-        <v>91</v>
-      </c>
-      <c r="G16" s="2" t="s">
-        <v>92</v>
-      </c>
-      <c r="H16" s="1" t="s">
-        <v>33</v>
-      </c>
       <c r="I16" s="1" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B17" s="1" t="s">
-        <v>94</v>
+        <v>37</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="D17" s="1" t="s">
-        <v>96</v>
+        <v>33</v>
       </c>
       <c r="E17" s="1" t="s">
-        <v>78</v>
+        <v>39</v>
       </c>
       <c r="F17" s="1" t="s">
         <v>97</v>
@@ -1108,91 +1191,88 @@
         <v>98</v>
       </c>
       <c r="H17" s="1" t="s">
-        <v>99</v>
+        <v>42</v>
       </c>
       <c r="I17" s="1" t="s">
-        <v>82</v>
+        <v>43</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B18" s="1" t="s">
-        <v>94</v>
+        <v>86</v>
       </c>
       <c r="C18" s="1" t="s">
+        <v>99</v>
+      </c>
+      <c r="D18" s="1" t="s">
+        <v>70</v>
+      </c>
+      <c r="E18" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="F18" s="1" t="s">
         <v>100</v>
       </c>
-      <c r="D18" s="1" t="s">
-        <v>96</v>
-      </c>
-      <c r="E18" s="1" t="s">
-        <v>78</v>
-      </c>
-      <c r="F18" s="1" t="s">
-        <v>97</v>
-      </c>
       <c r="G18" s="2" t="s">
-        <v>98</v>
+        <v>101</v>
       </c>
       <c r="H18" s="1" t="s">
+        <v>102</v>
+      </c>
+      <c r="I18" s="1" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B19" s="1" t="s">
+        <v>86</v>
+      </c>
+      <c r="C19" s="1" t="s">
         <v>99</v>
       </c>
-      <c r="I18" s="1" t="s">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="1" t="s">
-        <v>101</v>
-      </c>
-      <c r="B19" s="1" t="s">
-        <v>102</v>
-      </c>
-      <c r="C19" s="1" t="s">
-        <v>103</v>
-      </c>
       <c r="D19" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="E19" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="F19" s="1" t="s">
         <v>104</v>
       </c>
-      <c r="E19" s="1" t="s">
+      <c r="G19" s="2" t="s">
         <v>105</v>
       </c>
-      <c r="F19" s="1" t="s">
+      <c r="H19" s="1" t="s">
         <v>106</v>
       </c>
-      <c r="G19" s="2" t="s">
+      <c r="I19" s="1" t="s">
         <v>107</v>
-      </c>
-      <c r="H19" s="1" t="s">
-        <v>108</v>
-      </c>
-      <c r="I19" s="1" t="s">
-        <v>109</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B20" s="1" t="s">
-        <v>12</v>
+        <v>108</v>
       </c>
       <c r="C20" s="1" t="s">
+        <v>109</v>
+      </c>
+      <c r="D20" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="E20" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="F20" s="1" t="s">
         <v>110</v>
       </c>
-      <c r="D20" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="E20" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="F20" s="1" t="s">
+      <c r="G20" s="2" t="s">
         <v>111</v>
       </c>
-      <c r="G20" s="2" t="s">
-        <v>112</v>
-      </c>
       <c r="H20" s="1" t="s">
-        <v>33</v>
+        <v>106</v>
       </c>
       <c r="I20" s="1" t="s">
-        <v>34</v>
+        <v>107</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1200,215 +1280,368 @@
         <v>12</v>
       </c>
       <c r="C21" s="1" t="s">
+        <v>112</v>
+      </c>
+      <c r="D21" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="E21" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="F21" s="1" t="s">
         <v>113</v>
       </c>
-      <c r="D21" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="E21" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="F21" s="1" t="s">
+      <c r="G21" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="H21" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="I21" s="1" t="s">
         <v>114</v>
-      </c>
-      <c r="G21" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="H21" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="I21" s="1" t="s">
-        <v>19</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B22" s="1" t="s">
-        <v>12</v>
+        <v>37</v>
       </c>
       <c r="C22" s="1" t="s">
         <v>115</v>
       </c>
       <c r="D22" s="1" t="s">
-        <v>29</v>
+        <v>59</v>
       </c>
       <c r="E22" s="1" t="s">
-        <v>30</v>
+        <v>60</v>
       </c>
       <c r="F22" s="1" t="s">
         <v>116</v>
       </c>
       <c r="G22" s="2" t="s">
-        <v>112</v>
+        <v>117</v>
       </c>
       <c r="H22" s="1" t="s">
-        <v>33</v>
+        <v>23</v>
       </c>
       <c r="I22" s="1" t="s">
-        <v>34</v>
+        <v>118</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="1" t="s">
-        <v>117</v>
-      </c>
       <c r="B23" s="1" t="s">
-        <v>94</v>
+        <v>119</v>
       </c>
       <c r="C23" s="1" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="D23" s="1" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="E23" s="1" t="s">
-        <v>120</v>
+        <v>15</v>
       </c>
       <c r="F23" s="1" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="G23" s="2" t="s">
-        <v>122</v>
+        <v>123</v>
+      </c>
+      <c r="H23" s="1" t="s">
+        <v>124</v>
       </c>
       <c r="I23" s="1" t="s">
-        <v>123</v>
+        <v>107</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B24" s="1" t="s">
-        <v>55</v>
+        <v>119</v>
       </c>
       <c r="C24" s="1" t="s">
+        <v>125</v>
+      </c>
+      <c r="D24" s="1" t="s">
+        <v>121</v>
+      </c>
+      <c r="E24" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="F24" s="1" t="s">
+        <v>122</v>
+      </c>
+      <c r="G24" s="2" t="s">
+        <v>123</v>
+      </c>
+      <c r="H24" s="1" t="s">
         <v>124</v>
       </c>
-      <c r="D24" s="1" t="s">
-        <v>125</v>
-      </c>
-      <c r="E24" s="1" t="s">
-        <v>78</v>
-      </c>
-      <c r="F24" s="1" t="s">
+      <c r="I24" s="1" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="1" t="s">
         <v>126</v>
       </c>
-      <c r="G24" s="2" t="s">
+      <c r="B25" s="1" t="s">
         <v>127</v>
       </c>
-      <c r="H24" s="1" t="s">
-        <v>99</v>
-      </c>
-      <c r="I24" s="1" t="s">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B25" s="1" t="s">
-        <v>55</v>
-      </c>
       <c r="C25" s="1" t="s">
-        <v>124</v>
+        <v>128</v>
       </c>
       <c r="D25" s="1" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="E25" s="1" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="F25" s="1" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="G25" s="2" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="H25" s="1" t="s">
-        <v>33</v>
+        <v>133</v>
       </c>
       <c r="I25" s="1" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B26" s="1" t="s">
-        <v>55</v>
+        <v>12</v>
       </c>
       <c r="C26" s="1" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="D26" s="1" t="s">
-        <v>125</v>
+        <v>45</v>
       </c>
       <c r="E26" s="1" t="s">
-        <v>78</v>
+        <v>46</v>
       </c>
       <c r="F26" s="1" t="s">
-        <v>126</v>
+        <v>136</v>
       </c>
       <c r="G26" s="2" t="s">
-        <v>127</v>
+        <v>137</v>
       </c>
       <c r="H26" s="1" t="s">
-        <v>99</v>
+        <v>23</v>
       </c>
       <c r="I26" s="1" t="s">
-        <v>82</v>
+        <v>49</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B27" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="C27" s="1" t="s">
+        <v>138</v>
+      </c>
+      <c r="D27" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="E27" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="F27" s="1" t="s">
+        <v>139</v>
+      </c>
+      <c r="G27" s="2" t="s">
         <v>55</v>
       </c>
-      <c r="C27" s="1" t="s">
-        <v>133</v>
-      </c>
-      <c r="D27" s="1" t="s">
-        <v>128</v>
-      </c>
-      <c r="E27" s="1" t="s">
-        <v>129</v>
-      </c>
-      <c r="F27" s="1" t="s">
-        <v>130</v>
-      </c>
-      <c r="G27" s="2" t="s">
-        <v>134</v>
-      </c>
       <c r="H27" s="1" t="s">
-        <v>33</v>
+        <v>56</v>
       </c>
       <c r="I27" s="1" t="s">
-        <v>132</v>
+        <v>57</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B28" s="1" t="s">
-        <v>55</v>
+        <v>12</v>
       </c>
       <c r="C28" s="1" t="s">
-        <v>135</v>
+        <v>140</v>
       </c>
       <c r="D28" s="1" t="s">
-        <v>125</v>
+        <v>45</v>
       </c>
       <c r="E28" s="1" t="s">
-        <v>78</v>
+        <v>46</v>
       </c>
       <c r="F28" s="1" t="s">
-        <v>126</v>
+        <v>141</v>
       </c>
       <c r="G28" s="2" t="s">
-        <v>127</v>
+        <v>137</v>
       </c>
       <c r="H28" s="1" t="s">
-        <v>99</v>
+        <v>23</v>
       </c>
       <c r="I28" s="1" t="s">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="1048571" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048572" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048573" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048574" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048575" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048576" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+        <v>49</v>
+      </c>
+    </row>
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A29" s="1" t="s">
+        <v>142</v>
+      </c>
+      <c r="B29" s="1" t="s">
+        <v>119</v>
+      </c>
+      <c r="C29" s="1" t="s">
+        <v>143</v>
+      </c>
+      <c r="D29" s="1" t="s">
+        <v>144</v>
+      </c>
+      <c r="E29" s="1" t="s">
+        <v>145</v>
+      </c>
+      <c r="F29" s="1" t="s">
+        <v>146</v>
+      </c>
+      <c r="G29" s="2" t="s">
+        <v>147</v>
+      </c>
+      <c r="I29" s="1" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B30" s="1" t="s">
+        <v>86</v>
+      </c>
+      <c r="C30" s="1" t="s">
+        <v>149</v>
+      </c>
+      <c r="D30" s="1" t="s">
+        <v>150</v>
+      </c>
+      <c r="E30" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="F30" s="1" t="s">
+        <v>151</v>
+      </c>
+      <c r="G30" s="2" t="s">
+        <v>152</v>
+      </c>
+      <c r="H30" s="1" t="s">
+        <v>124</v>
+      </c>
+      <c r="I30" s="1" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B31" s="1" t="s">
+        <v>86</v>
+      </c>
+      <c r="C31" s="1" t="s">
+        <v>149</v>
+      </c>
+      <c r="D31" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="E31" s="1" t="s">
+        <v>153</v>
+      </c>
+      <c r="F31" s="1" t="s">
+        <v>154</v>
+      </c>
+      <c r="G31" s="2" t="s">
+        <v>155</v>
+      </c>
+      <c r="H31" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="I31" s="1" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B32" s="1" t="s">
+        <v>86</v>
+      </c>
+      <c r="C32" s="1" t="s">
+        <v>157</v>
+      </c>
+      <c r="D32" s="1" t="s">
+        <v>150</v>
+      </c>
+      <c r="E32" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="F32" s="1" t="s">
+        <v>151</v>
+      </c>
+      <c r="G32" s="2" t="s">
+        <v>152</v>
+      </c>
+      <c r="H32" s="1" t="s">
+        <v>124</v>
+      </c>
+      <c r="I32" s="1" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B33" s="1" t="s">
+        <v>86</v>
+      </c>
+      <c r="C33" s="1" t="s">
+        <v>157</v>
+      </c>
+      <c r="D33" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="E33" s="1" t="s">
+        <v>153</v>
+      </c>
+      <c r="F33" s="1" t="s">
+        <v>154</v>
+      </c>
+      <c r="G33" s="2" t="s">
+        <v>158</v>
+      </c>
+      <c r="H33" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="I33" s="1" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B34" s="1" t="s">
+        <v>86</v>
+      </c>
+      <c r="C34" s="1" t="s">
+        <v>159</v>
+      </c>
+      <c r="D34" s="1" t="s">
+        <v>150</v>
+      </c>
+      <c r="E34" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="F34" s="1" t="s">
+        <v>151</v>
+      </c>
+      <c r="G34" s="2" t="s">
+        <v>152</v>
+      </c>
+      <c r="H34" s="1" t="s">
+        <v>124</v>
+      </c>
+      <c r="I34" s="1" t="s">
+        <v>107</v>
+      </c>
+    </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>